<commit_message>
feat: add store-level DIWA rollout tracking and improve Gantt PDF reporting
</commit_message>
<xml_diff>
--- a/References/Hybrid SDLC Agile Templates/DBS - LINK HUB - Hybrid SDLC Agile.xlsx
+++ b/References/Hybrid SDLC Agile Templates/DBS - LINK HUB - Hybrid SDLC Agile.xlsx
@@ -21,7 +21,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" uniqueCount="205">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" uniqueCount="207">
   <si>
     <t>Template Name</t>
   </si>
@@ -486,6 +486,12 @@
   </si>
   <si>
     <t>Use the matrix as the cross-department reporting view. Milestone marks the primary owning department and Waiting is the recommended initial state; replace these with current status or target week as planning progresses. Imported Sub-Tasks remain the source of progress percentages.</t>
+  </si>
+  <si>
+    <t>Parallel planning</t>
+  </si>
+  <si>
+    <t>Independent departmental readiness checkpoints run in parallel after the target workflow is approved. LINK HUB business processes also run as parallel workstreams; design/build/QA/UAT/release gates inside each process remain sequential.</t>
   </si>
   <si>
     <t>Task Board</t>
@@ -5338,8 +5344,12 @@
       </c>
     </row>
     <row r="14" spans="1:2">
-      <c r="A14" s="2"/>
-      <c r="B14" s="2"/>
+      <c r="A14" s="2" t="s">
+        <v>167</v>
+      </c>
+      <c r="B14" s="2" t="s">
+        <v>168</v>
+      </c>
     </row>
     <row r="15" spans="1:2">
       <c r="A15" s="2"/>
@@ -6108,7 +6118,7 @@
   <sheetData>
     <row r="1" spans="1:4">
       <c r="A1" s="4" t="s">
-        <v>167</v>
+        <v>169</v>
       </c>
       <c r="B1" s="4"/>
       <c r="C1" s="4"/>
@@ -6116,30 +6126,30 @@
     </row>
     <row r="2" spans="1:4">
       <c r="A2" s="2" t="s">
-        <v>168</v>
+        <v>170</v>
       </c>
       <c r="B2" s="2" t="s">
-        <v>169</v>
+        <v>171</v>
       </c>
       <c r="C2" s="2" t="s">
-        <v>170</v>
+        <v>172</v>
       </c>
       <c r="D2" s="2" t="s">
-        <v>171</v>
+        <v>173</v>
       </c>
     </row>
     <row r="3" spans="1:4">
       <c r="A3" s="2" t="s">
-        <v>172</v>
+        <v>174</v>
       </c>
       <c r="B3" s="2" t="s">
-        <v>173</v>
+        <v>175</v>
       </c>
       <c r="C3" s="2" t="s">
-        <v>174</v>
+        <v>176</v>
       </c>
       <c r="D3" s="2" t="s">
-        <v>175</v>
+        <v>177</v>
       </c>
     </row>
     <row r="4" spans="1:4">
@@ -6147,13 +6157,13 @@
         <v>10</v>
       </c>
       <c r="B4" s="2" t="s">
-        <v>176</v>
+        <v>178</v>
       </c>
       <c r="C4" s="2" t="s">
-        <v>177</v>
+        <v>179</v>
       </c>
       <c r="D4" s="2" t="s">
-        <v>178</v>
+        <v>180</v>
       </c>
     </row>
     <row r="5" spans="1:4">
@@ -6161,41 +6171,41 @@
         <v>8</v>
       </c>
       <c r="B5" s="2" t="s">
-        <v>179</v>
+        <v>181</v>
       </c>
       <c r="C5" s="2" t="s">
-        <v>180</v>
+        <v>182</v>
       </c>
       <c r="D5" s="2" t="s">
-        <v>181</v>
+        <v>183</v>
       </c>
     </row>
     <row r="6" spans="1:4">
       <c r="A6" s="2" t="s">
-        <v>182</v>
+        <v>184</v>
       </c>
       <c r="B6" s="2" t="s">
-        <v>183</v>
+        <v>185</v>
       </c>
       <c r="C6" s="2" t="s">
-        <v>184</v>
+        <v>186</v>
       </c>
       <c r="D6" s="2" t="s">
-        <v>185</v>
+        <v>187</v>
       </c>
     </row>
     <row r="7" spans="1:4">
       <c r="A7" s="2" t="s">
-        <v>155</v>
+        <v>157</v>
       </c>
       <c r="B7" s="2" t="s">
-        <v>186</v>
+        <v>188</v>
       </c>
       <c r="C7" s="2" t="s">
-        <v>187</v>
+        <v>189</v>
       </c>
       <c r="D7" s="2" t="s">
-        <v>188</v>
+        <v>190</v>
       </c>
     </row>
     <row r="8" spans="1:4">
@@ -7376,36 +7386,36 @@
   <sheetData>
     <row r="1" spans="1:6">
       <c r="A1" t="s">
-        <v>189</v>
+        <v>191</v>
       </c>
       <c r="B1" t="s">
-        <v>190</v>
+        <v>192</v>
       </c>
       <c r="C1" t="s">
-        <v>191</v>
+        <v>193</v>
       </c>
       <c r="D1" t="s">
-        <v>192</v>
+        <v>194</v>
       </c>
       <c r="E1" t="s">
-        <v>193</v>
+        <v>195</v>
       </c>
       <c r="F1" t="s">
-        <v>194</v>
+        <v>196</v>
       </c>
     </row>
     <row r="2" spans="1:6">
       <c r="A2" t="s">
-        <v>195</v>
+        <v>197</v>
       </c>
       <c r="B2" t="s">
-        <v>196</v>
+        <v>198</v>
       </c>
       <c r="C2" t="s">
-        <v>197</v>
+        <v>199</v>
       </c>
       <c r="D2" t="s">
-        <v>198</v>
+        <v>200</v>
       </c>
       <c r="E2" t="s">
         <v>33</v>
@@ -7419,27 +7429,27 @@
         <v>27</v>
       </c>
       <c r="B3" t="s">
-        <v>199</v>
+        <v>201</v>
       </c>
       <c r="C3" t="s">
-        <v>200</v>
+        <v>202</v>
       </c>
       <c r="D3" t="s">
-        <v>201</v>
+        <v>203</v>
       </c>
       <c r="E3" t="s">
-        <v>159</v>
+        <v>161</v>
       </c>
       <c r="F3" t="s">
-        <v>202</v>
+        <v>204</v>
       </c>
     </row>
     <row r="4" spans="1:6">
       <c r="B4" t="s">
-        <v>203</v>
+        <v>205</v>
       </c>
       <c r="C4" t="s">
-        <v>204</v>
+        <v>206</v>
       </c>
       <c r="D4" t="s">
         <v>30</v>

</xml_diff>